<commit_message>
Auditoría: validaciones de proforma y separación, venta al contado y saldo de inicial en cobranza
- La inicial de un plan financiado llega como máximo a 90% (100% generaba cuotas de S/ 0).
- No se emite proforma sin precio ni separación de S/ 0 o mayor al precio final.
- La venta al contado se registra (antes no contaba como venta) y la cobranza incluye el saldo
  de la inicial a la firma; etiquetas y recordatorios lo nombran correctamente.
- Web: el celular del formulario acepta el prefijo +51.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SuYMBC9vy1hrR2C5YCk9db
</commit_message>
<xml_diff>
--- a/entregables/software/ejemplos-excel/ejemplo-control-de-cobranza.xlsx
+++ b/entregables/software/ejemplos-excel/ejemplo-control-de-cobranza.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="48">
   <si>
     <t>CONTROL DE COBRANZA</t>
   </si>
@@ -70,10 +70,16 @@
     <t>Mz B Lt 3</t>
   </si>
   <si>
+    <t>Saldo de inicial</t>
+  </si>
+  <si>
+    <t>Pagada · 25/10/2026</t>
+  </si>
+  <si>
     <t>1 de 24</t>
   </si>
   <si>
-    <t>Pagada · 25/10/2026</t>
+    <t>Próxima (30 días)</t>
   </si>
   <si>
     <t>2 de 24</t>
@@ -767,7 +773,7 @@
     <tabColor rgb="FF0A3856"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr defaultRowHeight="18" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -835,15 +841,15 @@
       </c>
       <c r="B8"/>
       <c r="C8" s="6">
-        <v>0</v>
+        <v>967</v>
       </c>
       <c r="D8"/>
       <c r="E8" s="6">
-        <v>967</v>
+        <v>4300</v>
       </c>
       <c r="F8"/>
       <c r="G8" s="6">
-        <v>22233</v>
+        <v>23200</v>
       </c>
       <c r="H8"/>
     </row>
@@ -875,7 +881,7 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="10">
-        <v>46336.5</v>
+        <v>46327.5</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>14</v>
@@ -893,7 +899,7 @@
         <v>18</v>
       </c>
       <c r="G11" s="13">
-        <v>967</v>
+        <v>4300</v>
       </c>
       <c r="H11" s="11" t="s">
         <v>19</v>
@@ -901,7 +907,7 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="14">
-        <v>46366.5</v>
+        <v>46336.5</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>14</v>
@@ -927,7 +933,7 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="18">
-        <v>46397.5</v>
+        <v>46366.5</v>
       </c>
       <c r="B13" s="19" t="s">
         <v>14</v>
@@ -948,12 +954,12 @@
         <v>967</v>
       </c>
       <c r="H13" s="19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="14">
-        <v>46428.5</v>
+        <v>46397.5</v>
       </c>
       <c r="B14" s="15" t="s">
         <v>14</v>
@@ -968,18 +974,18 @@
         <v>17</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G14" s="17">
         <v>967</v>
       </c>
       <c r="H14" s="15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="18">
-        <v>46456.5</v>
+        <v>46428.5</v>
       </c>
       <c r="B15" s="19" t="s">
         <v>14</v>
@@ -994,18 +1000,18 @@
         <v>17</v>
       </c>
       <c r="F15" s="20" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G15" s="21">
         <v>967</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="14">
-        <v>46487.5</v>
+        <v>46456.5</v>
       </c>
       <c r="B16" s="15" t="s">
         <v>14</v>
@@ -1020,18 +1026,18 @@
         <v>17</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G16" s="17">
         <v>967</v>
       </c>
       <c r="H16" s="15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="18">
-        <v>46517.5</v>
+        <v>46487.5</v>
       </c>
       <c r="B17" s="19" t="s">
         <v>14</v>
@@ -1046,18 +1052,18 @@
         <v>17</v>
       </c>
       <c r="F17" s="20" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G17" s="21">
         <v>967</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="14">
-        <v>46548.5</v>
+        <v>46517.5</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>14</v>
@@ -1072,18 +1078,18 @@
         <v>17</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G18" s="17">
         <v>967</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="18">
-        <v>46578.5</v>
+        <v>46548.5</v>
       </c>
       <c r="B19" s="19" t="s">
         <v>14</v>
@@ -1098,18 +1104,18 @@
         <v>17</v>
       </c>
       <c r="F19" s="20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G19" s="21">
         <v>967</v>
       </c>
       <c r="H19" s="19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="14">
-        <v>46609.5</v>
+        <v>46578.5</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>14</v>
@@ -1124,18 +1130,18 @@
         <v>17</v>
       </c>
       <c r="F20" s="16" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G20" s="17">
         <v>967</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="18">
-        <v>46640.5</v>
+        <v>46609.5</v>
       </c>
       <c r="B21" s="19" t="s">
         <v>14</v>
@@ -1150,18 +1156,18 @@
         <v>17</v>
       </c>
       <c r="F21" s="20" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G21" s="21">
         <v>967</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="14">
-        <v>46670.5</v>
+        <v>46640.5</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>14</v>
@@ -1176,18 +1182,18 @@
         <v>17</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G22" s="17">
         <v>967</v>
       </c>
       <c r="H22" s="15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="18">
-        <v>46701.5</v>
+        <v>46670.5</v>
       </c>
       <c r="B23" s="19" t="s">
         <v>14</v>
@@ -1202,18 +1208,18 @@
         <v>17</v>
       </c>
       <c r="F23" s="20" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G23" s="21">
         <v>967</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="14">
-        <v>46731.5</v>
+        <v>46701.5</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>14</v>
@@ -1228,18 +1234,18 @@
         <v>17</v>
       </c>
       <c r="F24" s="16" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G24" s="17">
         <v>967</v>
       </c>
       <c r="H24" s="15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="18">
-        <v>46762.5</v>
+        <v>46731.5</v>
       </c>
       <c r="B25" s="19" t="s">
         <v>14</v>
@@ -1254,18 +1260,18 @@
         <v>17</v>
       </c>
       <c r="F25" s="20" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G25" s="21">
         <v>967</v>
       </c>
       <c r="H25" s="19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="14">
-        <v>46793.5</v>
+        <v>46762.5</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>14</v>
@@ -1280,18 +1286,18 @@
         <v>17</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G26" s="17">
         <v>967</v>
       </c>
       <c r="H26" s="15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="18">
-        <v>46822.5</v>
+        <v>46793.5</v>
       </c>
       <c r="B27" s="19" t="s">
         <v>14</v>
@@ -1306,18 +1312,18 @@
         <v>17</v>
       </c>
       <c r="F27" s="20" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G27" s="21">
         <v>967</v>
       </c>
       <c r="H27" s="19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="14">
-        <v>46853.5</v>
+        <v>46822.5</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>14</v>
@@ -1332,18 +1338,18 @@
         <v>17</v>
       </c>
       <c r="F28" s="16" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G28" s="17">
         <v>967</v>
       </c>
       <c r="H28" s="15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="18">
-        <v>46883.5</v>
+        <v>46853.5</v>
       </c>
       <c r="B29" s="19" t="s">
         <v>14</v>
@@ -1358,18 +1364,18 @@
         <v>17</v>
       </c>
       <c r="F29" s="20" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G29" s="21">
         <v>967</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="14">
-        <v>46914.5</v>
+        <v>46883.5</v>
       </c>
       <c r="B30" s="15" t="s">
         <v>14</v>
@@ -1384,18 +1390,18 @@
         <v>17</v>
       </c>
       <c r="F30" s="16" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G30" s="17">
         <v>967</v>
       </c>
       <c r="H30" s="15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="18">
-        <v>46944.5</v>
+        <v>46914.5</v>
       </c>
       <c r="B31" s="19" t="s">
         <v>14</v>
@@ -1410,18 +1416,18 @@
         <v>17</v>
       </c>
       <c r="F31" s="20" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G31" s="21">
         <v>967</v>
       </c>
       <c r="H31" s="19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="14">
-        <v>46975.5</v>
+        <v>46944.5</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>14</v>
@@ -1436,18 +1442,18 @@
         <v>17</v>
       </c>
       <c r="F32" s="16" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G32" s="17">
         <v>967</v>
       </c>
       <c r="H32" s="15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="18">
-        <v>47006.5</v>
+        <v>46975.5</v>
       </c>
       <c r="B33" s="19" t="s">
         <v>14</v>
@@ -1462,69 +1468,95 @@
         <v>17</v>
       </c>
       <c r="F33" s="20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G33" s="21">
         <v>967</v>
       </c>
       <c r="H33" s="19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="14">
+        <v>47006.5</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="E34" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F34" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="G34" s="17">
+        <v>967</v>
+      </c>
+      <c r="H34" s="15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="18">
         <v>47036.5</v>
       </c>
-      <c r="B34" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="C34" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="D34" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="E34" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="F34" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="G34" s="17">
+      <c r="B35" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="D35" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="E35" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F35" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="G35" s="21">
         <v>959</v>
       </c>
-      <c r="H34" s="15" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="35" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="B35" s="22"/>
-      <c r="C35" s="22"/>
-      <c r="D35" s="22"/>
-      <c r="E35" s="22"/>
-      <c r="F35" s="22"/>
-      <c r="G35" s="23">
-        <f>SUBTOTAL(9,G11:G34)</f>
-      </c>
-      <c r="H35" s="22"/>
-    </row>
-    <row r="37" ht="42" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="B37"/>
-      <c r="C37"/>
-      <c r="D37"/>
-      <c r="E37"/>
-      <c r="F37"/>
-      <c r="G37"/>
-      <c r="H37"/>
+      <c r="H35" s="19" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="B36" s="22"/>
+      <c r="C36" s="22"/>
+      <c r="D36" s="22"/>
+      <c r="E36" s="22"/>
+      <c r="F36" s="22"/>
+      <c r="G36" s="23">
+        <f>SUBTOTAL(9,G11:G35)</f>
+      </c>
+      <c r="H36" s="22"/>
+    </row>
+    <row r="38" ht="42" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B38"/>
+      <c r="C38"/>
+      <c r="D38"/>
+      <c r="E38"/>
+      <c r="F38"/>
+      <c r="G38"/>
+      <c r="H38"/>
     </row>
   </sheetData>
-  <autoFilter ref="A10:H34"/>
+  <autoFilter ref="A10:H35"/>
   <mergeCells count="11">
     <mergeCell ref="C2:H2"/>
     <mergeCell ref="C3:H3"/>
@@ -1536,7 +1568,7 @@
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="E8:F8"/>
     <mergeCell ref="G8:H8"/>
-    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A38:H38"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.2" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>